<commit_message>
More cleaning up refactoring.
-- eliminated duplicated buildingData fields in several classes and subclass.  All inherit from the WindLoadCalculator base class.
-- cleaned up ComputeEffectiveWindAreas by making it parameterless since the subclasses already know all of the arguments we were passing to it.
</commit_message>
<xml_diff>
--- a/WindLoadCalculations/ClassInheritanceSummary.xlsx
+++ b/WindLoadCalculations/ClassInheritanceSummary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\ShearWallCalculator\WindLoadCalculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F15AC2-A52E-427D-A501-45581D2292DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D0F6CC7-1BFE-4636-94CD-54428195D91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28320" yWindow="975" windowWidth="25125" windowHeight="14130" xr2:uid="{22411508-42AA-4A47-BA84-DFEA7F97E3DA}"/>
+    <workbookView xWindow="-26550" yWindow="555" windowWidth="25125" windowHeight="14130" xr2:uid="{22411508-42AA-4A47-BA84-DFEA7F97E3DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="65">
   <si>
     <t>WindLoadCalculator_Base</t>
   </si>
@@ -62,6 +62,12 @@
     <t>AreaCalculator_ASCE7_22_Base</t>
   </si>
   <si>
+    <t>AreaCalculator_CC_ASCE7_22_Base</t>
+  </si>
+  <si>
+    <t>AreaCalculator_MWFRS_ASCE7_22_Base</t>
+  </si>
+  <si>
     <t>AreaCalculator_CC_ASCE7_16_Base</t>
   </si>
   <si>
@@ -174,13 +180,64 @@
   </si>
   <si>
     <t>abstract GetGCpi</t>
+  </si>
+  <si>
+    <t>CalcDynamicWind</t>
+  </si>
+  <si>
+    <t>CalcExternalPress</t>
+  </si>
+  <si>
+    <t>CalcNetPress</t>
+  </si>
+  <si>
+    <t>buildingData</t>
+  </si>
+  <si>
+    <t>Parameters</t>
+  </si>
+  <si>
+    <t>abstract buildingData</t>
+  </si>
+  <si>
+    <t>effWindAreas</t>
+  </si>
+  <si>
+    <t>abstract ComputeEffectiveWindAreas</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>abstract CritDim_a</t>
+  </si>
+  <si>
+    <t>abstract HasCritDim</t>
+  </si>
+  <si>
+    <t>ComputeEffectiveWindAreas</t>
+  </si>
+  <si>
+    <t>hasCritDim = false</t>
+  </si>
+  <si>
+    <t>Critdim_a = 0</t>
+  </si>
+  <si>
+    <t>hasCritDim = true;</t>
+  </si>
+  <si>
+    <t>CritDim_a = ComputeCritDim()</t>
+  </si>
+  <si>
+    <t>ComputeEffectiveWindAreas()</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,13 +245,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -209,9 +293,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -549,236 +638,350 @@
   <dimension ref="A2:Q54"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="2" spans="2:17">
-      <c r="B2" t="s">
+    <row r="2" spans="2:11" ht="15">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="K2" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:17">
+    <row r="3" spans="2:11">
       <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11">
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11">
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="15">
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11">
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+      <c r="K7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11">
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" t="s">
+        <v>42</v>
+      </c>
+      <c r="K8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11">
+      <c r="B9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="2:11">
+      <c r="B10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="14" spans="2:11" ht="15">
+      <c r="F14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="K14" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="2:17">
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="2:17">
-      <c r="B5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="2:17">
-      <c r="B6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17">
-      <c r="B7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="2:17">
-      <c r="B8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17">
-      <c r="F11" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q11" t="s">
+    </row>
+    <row r="15" spans="2:11">
+      <c r="F15" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="12" spans="2:17">
-      <c r="F12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="2:17">
-      <c r="F13" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q13" t="s">
+      <c r="K15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11">
+      <c r="F16" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="14" spans="2:17">
-      <c r="F14" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="2:17">
-      <c r="B16" t="s">
-        <v>36</v>
+      <c r="K16" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
+      <c r="F18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="15">
+      <c r="F19" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17">
-      <c r="B18" s="1" t="s">
+      <c r="K19" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="15">
+      <c r="B20" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="K20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17">
+      <c r="B21" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="21" spans="1:17">
-      <c r="B21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17">
-      <c r="B24" s="1"/>
-    </row>
-    <row r="25" spans="1:17">
-      <c r="B25" s="1"/>
+      <c r="K21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17">
+      <c r="B22" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="15">
+      <c r="B25" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="26" spans="1:17">
       <c r="B26" s="1"/>
     </row>
     <row r="30" spans="1:17">
       <c r="Q30" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="1:17">
       <c r="Q31" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17">
-      <c r="B32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="15">
+      <c r="B32" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H32" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="L32" t="s">
+      <c r="I32" s="3"/>
+      <c r="L32" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="2:17">
+      <c r="B33" t="s">
+        <v>54</v>
+      </c>
+      <c r="H33" t="s">
+        <v>61</v>
+      </c>
+      <c r="L33" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="2:17">
+      <c r="B34" t="s">
+        <v>57</v>
+      </c>
+      <c r="H34" t="s">
+        <v>60</v>
+      </c>
+      <c r="L34" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="2:17">
+      <c r="B35" t="s">
+        <v>58</v>
+      </c>
+      <c r="H35" t="s">
+        <v>59</v>
+      </c>
+      <c r="L35" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="2:17">
+      <c r="B36" t="s">
+        <v>56</v>
+      </c>
+      <c r="H36" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="2:17" ht="15">
+      <c r="B37" t="s">
+        <v>53</v>
+      </c>
+      <c r="L37" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="2:17">
+      <c r="B38" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="2:17">
+      <c r="Q39" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="2:17">
+      <c r="Q40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="2:17">
+      <c r="Q44" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="45" spans="2:17">
+      <c r="Q45" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46" spans="2:17" ht="15">
+      <c r="H46" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L46" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="Q32" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="33" spans="8:17">
-      <c r="Q33" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="34" spans="8:17">
-      <c r="Q34" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="36" spans="8:17">
-      <c r="Q36" t="s">
+      <c r="Q46" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47" spans="2:17">
+      <c r="H47" t="s">
+        <v>61</v>
+      </c>
+      <c r="L47" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q47" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="8:17">
-      <c r="L37" t="s">
+    <row r="48" spans="2:17">
+      <c r="H48" t="s">
+        <v>60</v>
+      </c>
+      <c r="L48" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="49" spans="8:17">
+      <c r="H49" t="s">
+        <v>59</v>
+      </c>
+      <c r="L49" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="8:17">
+      <c r="H50" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="51" spans="8:17">
+      <c r="Q51" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="52" spans="8:17" ht="15">
+      <c r="L52" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q37" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="38" spans="8:17">
-      <c r="Q38" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="39" spans="8:17">
-      <c r="Q39" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="40" spans="8:17">
-      <c r="Q40" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" spans="8:17">
-      <c r="Q44" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="45" spans="8:17">
-      <c r="Q45" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="46" spans="8:17">
-      <c r="H46" t="s">
-        <v>7</v>
-      </c>
-      <c r="L46" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q46" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="47" spans="8:17">
-      <c r="Q47" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="48" spans="8:17">
-      <c r="Q48" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="50" spans="12:17">
-      <c r="Q50" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="51" spans="12:17">
-      <c r="Q51" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="52" spans="12:17">
-      <c r="L52" t="s">
-        <v>9</v>
-      </c>
       <c r="Q52" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="53" spans="12:17">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="53" spans="8:17">
       <c r="Q53" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="54" spans="12:17">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" spans="8:17">
       <c r="Q54" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More polymorphism fixes for Chapter 30 figures.
-  Added Curves for Figure 27.3-1 for MWFRS of ASCE 7-16
</commit_message>
<xml_diff>
--- a/WindLoadCalculations/ClassInheritanceSummary.xlsx
+++ b/WindLoadCalculations/ClassInheritanceSummary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\ShearWallCalculator\WindLoadCalculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D0F6CC7-1BFE-4636-94CD-54428195D91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E500CE5-3E00-42DF-81D2-7AF372AAAD13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-26550" yWindow="555" windowWidth="25125" windowHeight="14130" xr2:uid="{22411508-42AA-4A47-BA84-DFEA7F97E3DA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="75">
   <si>
     <t>WindLoadCalculator_Base</t>
   </si>
@@ -231,6 +231,36 @@
   </si>
   <si>
     <t>ComputeEffectiveWindAreas()</t>
+  </si>
+  <si>
+    <t>CritDim_a = 0</t>
+  </si>
+  <si>
+    <t>hasCritDim = false;</t>
+  </si>
+  <si>
+    <t>IsValidRectangle</t>
+  </si>
+  <si>
+    <t>extGcpCurve_roof</t>
+  </si>
+  <si>
+    <t>extGCpCurve_wall</t>
+  </si>
+  <si>
+    <t>Cp_WW</t>
+  </si>
+  <si>
+    <t>Cp_LW</t>
+  </si>
+  <si>
+    <t>Cp_SW</t>
+  </si>
+  <si>
+    <t>CpCurve_roof</t>
+  </si>
+  <si>
+    <t>CpCurve_wall</t>
   </si>
 </sst>
 </file>
@@ -635,7 +665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B465602-C2A7-405C-BCBF-2E4928F7F3E2}">
-  <dimension ref="A2:Q54"/>
+  <dimension ref="A2:T55"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="2" spans="2:11" ht="15">
@@ -678,16 +708,19 @@
       <c r="F5" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="6" spans="2:11" ht="15">
+      <c r="K5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11">
       <c r="B6" t="s">
         <v>40</v>
       </c>
       <c r="F6" t="s">
         <v>48</v>
       </c>
-      <c r="K6" s="6" t="s">
-        <v>2</v>
+      <c r="K6" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="2:11">
@@ -697,9 +730,6 @@
       <c r="F7" t="s">
         <v>41</v>
       </c>
-      <c r="K7" t="s">
-        <v>49</v>
-      </c>
     </row>
     <row r="8" spans="2:11">
       <c r="B8" t="s">
@@ -708,28 +738,46 @@
       <c r="F8" t="s">
         <v>42</v>
       </c>
-      <c r="K8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11">
+    </row>
+    <row r="9" spans="2:11" ht="15">
       <c r="B9" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C9" s="2"/>
+      <c r="K9" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" spans="2:11">
       <c r="B10" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C10" s="2"/>
+      <c r="K10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11">
+      <c r="K11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11">
+      <c r="K12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11">
+      <c r="K13" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="14" spans="2:11" ht="15">
       <c r="F14" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="K14" s="5" t="s">
-        <v>34</v>
+      <c r="K14" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="2:11">
@@ -737,7 +785,7 @@
         <v>32</v>
       </c>
       <c r="K15" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="2:11">
@@ -745,10 +793,10 @@
         <v>33</v>
       </c>
       <c r="K16" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20">
       <c r="A17" s="1" t="s">
         <v>44</v>
       </c>
@@ -756,20 +804,20 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" spans="1:20">
       <c r="F18" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="15">
+    <row r="19" spans="1:20" ht="15">
       <c r="F19" t="s">
         <v>42</v>
       </c>
-      <c r="K19" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" ht="15">
+      <c r="K19" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" ht="15">
       <c r="B20" s="5" t="s">
         <v>38</v>
       </c>
@@ -777,7 +825,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:20">
       <c r="B21" s="1" t="s">
         <v>43</v>
       </c>
@@ -785,30 +833,51 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:20">
       <c r="B22" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="15">
+    <row r="24" spans="1:20" ht="15">
+      <c r="K24" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" ht="15">
       <c r="B25" s="6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="26" spans="1:17">
+      <c r="K25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20">
       <c r="B26" s="1"/>
-    </row>
-    <row r="30" spans="1:17">
+      <c r="K26" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20">
+      <c r="T28" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20">
+      <c r="T29" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20">
       <c r="Q30" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:17">
+    <row r="31" spans="1:20">
       <c r="Q31" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="15">
+    <row r="32" spans="1:20" ht="15">
       <c r="B32" s="4" t="s">
         <v>3</v>
       </c>
@@ -888,16 +957,25 @@
       <c r="B38" t="s">
         <v>55</v>
       </c>
+      <c r="L38" t="s">
+        <v>65</v>
+      </c>
       <c r="Q38" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="39" spans="2:17">
+      <c r="L39" t="s">
+        <v>66</v>
+      </c>
       <c r="Q39" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="40" spans="2:17">
+      <c r="L40" t="s">
+        <v>64</v>
+      </c>
       <c r="Q40" t="s">
         <v>15</v>
       </c>
@@ -975,13 +1053,24 @@
       </c>
     </row>
     <row r="53" spans="8:17">
+      <c r="L53" t="s">
+        <v>65</v>
+      </c>
       <c r="Q53" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="54" spans="8:17">
+      <c r="L54" t="s">
+        <v>66</v>
+      </c>
       <c r="Q54" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="55" spans="8:17">
+      <c r="L55" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More refactoring and work on MWFRS for Gables and Hips
</commit_message>
<xml_diff>
--- a/WindLoadCalculations/ClassInheritanceSummary.xlsx
+++ b/WindLoadCalculations/ClassInheritanceSummary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\ShearWallCalculator\WindLoadCalculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F4F395-E6B8-494B-AEA3-1339036ED891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD763267-2206-419D-9D11-D9A72E56C1E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26550" yWindow="555" windowWidth="25125" windowHeight="14130" xr2:uid="{22411508-42AA-4A47-BA84-DFEA7F97E3DA}"/>
+    <workbookView xWindow="1920" yWindow="840" windowWidth="25125" windowHeight="14130" xr2:uid="{22411508-42AA-4A47-BA84-DFEA7F97E3DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="76">
   <si>
     <t>WindLoadCalculator_Base</t>
   </si>
@@ -261,6 +261,9 @@
   </si>
   <si>
     <t>CpCurve_wall</t>
+  </si>
+  <si>
+    <t>CalculatePressure</t>
   </si>
 </sst>
 </file>
@@ -323,10 +326,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -669,13 +671,13 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="2" spans="2:11" ht="15">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
@@ -740,24 +742,25 @@
       </c>
     </row>
     <row r="9" spans="2:11" ht="15">
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="2:11">
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="2"/>
       <c r="K10" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="2:11">
+      <c r="B11" t="s">
+        <v>75</v>
+      </c>
       <c r="K11" t="s">
         <v>50</v>
       </c>
@@ -773,7 +776,7 @@
       </c>
     </row>
     <row r="14" spans="2:11" ht="15">
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="3" t="s">
         <v>5</v>
       </c>
       <c r="K14" t="s">
@@ -813,12 +816,12 @@
       <c r="F19" t="s">
         <v>42</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="K19" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:20" ht="15">
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>38</v>
       </c>
       <c r="K20" t="s">
@@ -839,12 +842,12 @@
       </c>
     </row>
     <row r="24" spans="1:20" ht="15">
-      <c r="K24" s="6" t="s">
+      <c r="K24" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:20" ht="15">
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="5" t="s">
         <v>39</v>
       </c>
       <c r="K25" t="s">
@@ -878,14 +881,14 @@
       </c>
     </row>
     <row r="32" spans="1:20" ht="15">
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H32" s="4" t="s">
+      <c r="H32" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I32" s="3"/>
-      <c r="L32" s="4" t="s">
+      <c r="I32" s="2"/>
+      <c r="L32" s="3" t="s">
         <v>10</v>
       </c>
       <c r="Q32" t="s">
@@ -946,7 +949,7 @@
       <c r="B37" t="s">
         <v>53</v>
       </c>
-      <c r="L37" s="4" t="s">
+      <c r="L37" s="3" t="s">
         <v>11</v>
       </c>
       <c r="Q37" t="s">
@@ -991,10 +994,10 @@
       </c>
     </row>
     <row r="46" spans="2:17" ht="15">
-      <c r="H46" s="4" t="s">
+      <c r="H46" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="L46" s="4" t="s">
+      <c r="L46" s="3" t="s">
         <v>8</v>
       </c>
       <c r="Q46" t="s">
@@ -1045,7 +1048,7 @@
       </c>
     </row>
     <row r="52" spans="8:17" ht="15">
-      <c r="L52" s="4" t="s">
+      <c r="L52" s="3" t="s">
         <v>9</v>
       </c>
       <c r="Q52" t="s">

</xml_diff>